<commit_message>
update floor weight spreadsheet
</commit_message>
<xml_diff>
--- a/Beaverton Creek Floor and Roof Unit Weights.xlsx
+++ b/Beaverton Creek Floor and Roof Unit Weights.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kpffla-my.sharepoint.com/personal/andy_sazima_kpff_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kpffla-my.sharepoint.com/personal/andy_sazima_kpff_com/Documents/Projects/Beaverton Creek/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1817464F-48AB-4F5A-9E10-BDAEE0550FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{1817464F-48AB-4F5A-9E10-BDAEE0550FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD3B5E41-3CE8-4CEA-B7FB-59DD1C958320}"/>
   <bookViews>
-    <workbookView xWindow="29160" yWindow="0" windowWidth="21600" windowHeight="15585" activeTab="1" xr2:uid="{C4BC4AC7-676F-493A-B346-EB7A9058A7D3}"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4BC4AC7-676F-493A-B346-EB7A9058A7D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Floor" sheetId="1" r:id="rId1"/>
@@ -1079,21 +1079,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:N120"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="1.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="1" customWidth="1"/>
-    <col min="4" max="12" width="9.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.7109375" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="3.7265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="1.7265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" style="1" customWidth="1"/>
+    <col min="4" max="12" width="9.1796875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.7265625" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="M2" s="8"/>
     </row>
-    <row r="3" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="9"/>
       <c r="G3" s="5" t="s">
         <v>3</v>
@@ -1131,12 +1131,12 @@
       </c>
       <c r="K3" s="24">
         <f ca="1">TODAY()</f>
-        <v>46150</v>
+        <v>46163</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="11"/>
     </row>
-    <row r="4" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="G4" s="5" t="s">
         <v>5</v>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="M4" s="8"/>
     </row>
-    <row r="5" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="14"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -1170,7 +1170,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
     </row>
-    <row r="6" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
       <c r="C6" s="18"/>
       <c r="D6" s="19"/>
@@ -1183,7 +1183,7 @@
       <c r="K6" s="4"/>
       <c r="M6" s="11"/>
     </row>
-    <row r="7" spans="2:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="9"/>
       <c r="C7" s="25" t="s">
         <v>9</v>
@@ -1192,7 +1192,7 @@
       <c r="E7" s="22"/>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="9"/>
       <c r="C8" s="22"/>
       <c r="D8" s="22"/>
@@ -1200,7 +1200,7 @@
       <c r="F8" s="22"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="9"/>
       <c r="C9" s="28" t="s">
         <v>10</v>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:14" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" ht="11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9"/>
       <c r="C10" s="29" t="s">
         <v>13</v>
@@ -1239,7 +1239,7 @@
       <c r="M10" s="11"/>
       <c r="N10" s="20"/>
     </row>
-    <row r="11" spans="2:14" ht="11.1" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:14" ht="11.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B11" s="9"/>
       <c r="C11" s="31" t="s">
         <v>12</v>
@@ -1255,7 +1255,7 @@
       <c r="H11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="9"/>
       <c r="C12" s="31" t="s">
         <v>17</v>
@@ -1271,7 +1271,7 @@
       <c r="M12" s="11"/>
       <c r="N12" s="20"/>
     </row>
-    <row r="13" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="9"/>
       <c r="C13" s="31" t="s">
         <v>18</v>
@@ -1290,7 +1290,7 @@
       <c r="M13" s="11"/>
       <c r="N13" s="20"/>
     </row>
-    <row r="14" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="9"/>
       <c r="C14" s="9" t="s">
         <v>19</v>
@@ -1305,7 +1305,7 @@
       <c r="M14" s="11"/>
       <c r="N14" s="20"/>
     </row>
-    <row r="15" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="9"/>
       <c r="C15" s="9" t="s">
         <v>20</v>
@@ -1323,13 +1323,13 @@
       <c r="M15" s="11"/>
       <c r="N15" s="20"/>
     </row>
-    <row r="16" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="9"/>
       <c r="C16" s="9" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>22</v>
@@ -1338,31 +1338,31 @@
       <c r="M16" s="11"/>
       <c r="N16" s="20"/>
     </row>
-    <row r="17" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="9"/>
       <c r="C17" s="32" t="s">
         <v>28</v>
       </c>
       <c r="D17" s="33">
         <f>SUM(D11:D16)</f>
-        <v>28.3</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="E17" s="15"/>
       <c r="F17" s="15"/>
       <c r="G17" s="15"/>
       <c r="H17" s="17"/>
       <c r="I17" s="35" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M17" s="11"/>
       <c r="N17" s="20"/>
     </row>
-    <row r="18" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="9"/>
       <c r="M18" s="11"/>
       <c r="N18" s="20"/>
     </row>
-    <row r="19" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="9"/>
       <c r="C19" s="28" t="s">
         <v>29</v>
@@ -1377,7 +1377,7 @@
       <c r="M19" s="11"/>
       <c r="N19" s="20"/>
     </row>
-    <row r="20" spans="2:14" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" ht="11.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="9"/>
       <c r="C20" s="29" t="s">
         <v>13</v>
@@ -1396,7 +1396,7 @@
       <c r="M20" s="11"/>
       <c r="N20" s="20"/>
     </row>
-    <row r="21" spans="2:14" ht="11.1" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:14" ht="11.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B21" s="9"/>
       <c r="C21" s="31" t="s">
         <v>12</v>
@@ -1413,7 +1413,7 @@
       <c r="M21" s="11"/>
       <c r="N21" s="20"/>
     </row>
-    <row r="22" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="9"/>
       <c r="C22" s="31" t="s">
         <v>17</v>
@@ -1429,7 +1429,7 @@
       <c r="M22" s="11"/>
       <c r="N22" s="20"/>
     </row>
-    <row r="23" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="9"/>
       <c r="C23" s="31" t="s">
         <v>18</v>
@@ -1448,7 +1448,7 @@
       <c r="M23" s="11"/>
       <c r="N23" s="20"/>
     </row>
-    <row r="24" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="9"/>
       <c r="C24" s="9" t="s">
         <v>31</v>
@@ -1466,7 +1466,7 @@
       <c r="M24" s="11"/>
       <c r="N24" s="20"/>
     </row>
-    <row r="25" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="9"/>
       <c r="C25" s="9" t="s">
         <v>20</v>
@@ -1484,7 +1484,7 @@
       <c r="M25" s="11"/>
       <c r="N25" s="20"/>
     </row>
-    <row r="26" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="9"/>
       <c r="C26" s="9" t="s">
         <v>21</v>
@@ -1499,7 +1499,7 @@
       <c r="M26" s="11"/>
       <c r="N26" s="20"/>
     </row>
-    <row r="27" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="9"/>
       <c r="C27" s="32" t="s">
         <v>28</v>
@@ -1518,185 +1518,185 @@
       <c r="M27" s="11"/>
       <c r="N27" s="20"/>
     </row>
-    <row r="28" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="9"/>
       <c r="M28" s="11"/>
       <c r="N28" s="20"/>
     </row>
-    <row r="29" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="9"/>
       <c r="C29" s="21"/>
       <c r="L29" s="22"/>
       <c r="M29" s="11"/>
       <c r="N29" s="20"/>
     </row>
-    <row r="30" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="9"/>
       <c r="D30" s="23"/>
       <c r="L30" s="22"/>
       <c r="M30" s="11"/>
       <c r="N30" s="20"/>
     </row>
-    <row r="31" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="9"/>
       <c r="L31" s="22"/>
       <c r="M31" s="11"/>
       <c r="N31" s="20"/>
     </row>
-    <row r="32" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="9"/>
       <c r="D32" s="21"/>
       <c r="L32" s="22"/>
       <c r="M32" s="11"/>
       <c r="N32" s="20"/>
     </row>
-    <row r="33" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="9"/>
       <c r="L33" s="22"/>
       <c r="M33" s="11"/>
       <c r="N33" s="20"/>
     </row>
-    <row r="34" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="9"/>
       <c r="L34" s="22"/>
       <c r="M34" s="11"/>
       <c r="N34" s="20"/>
     </row>
-    <row r="35" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="9"/>
       <c r="L35" s="22"/>
       <c r="M35" s="11"/>
     </row>
-    <row r="36" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="9"/>
       <c r="L36" s="22"/>
       <c r="M36" s="11"/>
     </row>
-    <row r="37" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="9"/>
       <c r="L37" s="22"/>
       <c r="M37" s="11"/>
     </row>
-    <row r="38" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="9"/>
       <c r="L38" s="22"/>
       <c r="M38" s="11"/>
     </row>
-    <row r="39" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="9"/>
       <c r="L39" s="22"/>
       <c r="M39" s="11"/>
     </row>
-    <row r="40" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="9"/>
       <c r="L40" s="22"/>
       <c r="M40" s="11"/>
     </row>
-    <row r="41" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="9"/>
       <c r="L41" s="22"/>
       <c r="M41" s="11"/>
     </row>
-    <row r="42" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="9"/>
       <c r="L42" s="22"/>
       <c r="M42" s="11"/>
     </row>
-    <row r="43" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="9"/>
       <c r="L43" s="22"/>
       <c r="M43" s="11"/>
     </row>
-    <row r="44" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="9"/>
       <c r="L44" s="22"/>
       <c r="M44" s="11"/>
     </row>
-    <row r="45" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="9"/>
       <c r="L45" s="22"/>
       <c r="M45" s="11"/>
     </row>
-    <row r="46" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="9"/>
       <c r="L46" s="22"/>
       <c r="M46" s="11"/>
     </row>
-    <row r="47" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="9"/>
       <c r="L47" s="22"/>
       <c r="M47" s="11"/>
     </row>
-    <row r="48" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="9"/>
       <c r="L48" s="22"/>
       <c r="M48" s="11"/>
     </row>
-    <row r="49" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="9"/>
       <c r="L49" s="22"/>
       <c r="M49" s="11"/>
     </row>
-    <row r="50" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="9"/>
       <c r="L50" s="22"/>
       <c r="M50" s="11"/>
     </row>
-    <row r="51" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="9"/>
       <c r="L51" s="22"/>
       <c r="M51" s="11"/>
     </row>
-    <row r="52" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="9"/>
       <c r="L52" s="22"/>
       <c r="M52" s="11"/>
     </row>
-    <row r="53" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="9"/>
       <c r="M53" s="11"/>
     </row>
-    <row r="54" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="9"/>
       <c r="M54" s="11"/>
     </row>
-    <row r="55" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="9"/>
       <c r="M55" s="11"/>
     </row>
-    <row r="56" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="9"/>
       <c r="M56" s="11"/>
     </row>
-    <row r="57" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="9"/>
       <c r="M57" s="11"/>
     </row>
-    <row r="58" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="9"/>
       <c r="M58" s="11"/>
     </row>
-    <row r="59" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="9"/>
       <c r="M59" s="11"/>
     </row>
-    <row r="60" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="9"/>
       <c r="M60" s="11"/>
     </row>
-    <row r="61" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="9"/>
       <c r="M61" s="11"/>
     </row>
-    <row r="62" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="9"/>
       <c r="M62" s="11"/>
     </row>
-    <row r="63" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="9"/>
       <c r="M63" s="11"/>
     </row>
-    <row r="64" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="14"/>
       <c r="C64" s="15"/>
       <c r="D64" s="15"/>
@@ -1710,62 +1710,62 @@
       <c r="L64" s="15"/>
       <c r="M64" s="17"/>
     </row>
-    <row r="65" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="67" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="68" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="69" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="70" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="73" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="74" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="76" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="77" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="78" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="80" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="81" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="82" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="83" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="85" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="87" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="89" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="90" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="91" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="92" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="94" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="103" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="104" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="105" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="106" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="107" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="108" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="109" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="110" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="111" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="112" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="113" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="114" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="115" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="116" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="117" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="118" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="119" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="120" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="65" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="83" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="84" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="110" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="111" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="113" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="114" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="115" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="116" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="117" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="118" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="119" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="120" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection formatCells="0" insertHyperlinks="0" sort="0" autoFilter="0" pivotTables="0"/>
   <conditionalFormatting sqref="L1">
@@ -1808,21 +1808,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:N109"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="10.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="1.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="1" customWidth="1"/>
-    <col min="4" max="12" width="9.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.7109375" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="3.7265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="1.7265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" style="1" customWidth="1"/>
+    <col min="4" max="12" width="9.1796875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.7265625" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="M2" s="8"/>
     </row>
-    <row r="3" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="9"/>
       <c r="G3" s="5" t="s">
         <v>3</v>
@@ -1860,12 +1860,12 @@
       </c>
       <c r="K3" s="24">
         <f ca="1">TODAY()</f>
-        <v>46150</v>
+        <v>46163</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="11"/>
     </row>
-    <row r="4" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="G4" s="5" t="s">
         <v>5</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="M4" s="8"/>
     </row>
-    <row r="5" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="14"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -1899,7 +1899,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="17"/>
     </row>
-    <row r="6" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
       <c r="C6" s="18"/>
       <c r="D6" s="19"/>
@@ -1912,7 +1912,7 @@
       <c r="K6" s="4"/>
       <c r="M6" s="11"/>
     </row>
-    <row r="7" spans="2:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="9"/>
       <c r="C7" s="25" t="s">
         <v>35</v>
@@ -1921,7 +1921,7 @@
       <c r="E7" s="22"/>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="9"/>
       <c r="C8" s="22"/>
       <c r="D8" s="22"/>
@@ -1929,7 +1929,7 @@
       <c r="F8" s="22"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="9"/>
       <c r="C9" s="28" t="s">
         <v>36</v>
@@ -1943,7 +1943,7 @@
       <c r="H9" s="8"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="2:14" ht="12" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" ht="11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="9"/>
       <c r="C10" s="29" t="s">
         <v>13</v>
@@ -1962,7 +1962,7 @@
       <c r="M10" s="11"/>
       <c r="N10" s="20"/>
     </row>
-    <row r="11" spans="2:14" ht="11.1" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:14" ht="11.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B11" s="9"/>
       <c r="C11" s="31" t="s">
         <v>38</v>
@@ -1975,7 +1975,7 @@
       <c r="H11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="9"/>
       <c r="C12" s="31" t="s">
         <v>39</v>
@@ -1996,7 +1996,7 @@
       <c r="M12" s="11"/>
       <c r="N12" s="20"/>
     </row>
-    <row r="13" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="9"/>
       <c r="C13" s="31" t="s">
         <v>42</v>
@@ -2010,7 +2010,7 @@
       <c r="M13" s="11"/>
       <c r="N13" s="20"/>
     </row>
-    <row r="14" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="9"/>
       <c r="C14" s="9" t="s">
         <v>43</v>
@@ -2031,7 +2031,7 @@
       <c r="M14" s="11"/>
       <c r="N14" s="20"/>
     </row>
-    <row r="15" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="9"/>
       <c r="C15" s="9" t="s">
         <v>57</v>
@@ -2048,7 +2048,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="9"/>
       <c r="C16" s="9" t="s">
         <v>20</v>
@@ -2066,7 +2066,7 @@
       <c r="M16" s="11"/>
       <c r="N16" s="20"/>
     </row>
-    <row r="17" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="9"/>
       <c r="C17" s="9" t="s">
         <v>21</v>
@@ -2081,7 +2081,7 @@
       <c r="M17" s="11"/>
       <c r="N17" s="20"/>
     </row>
-    <row r="18" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="9"/>
       <c r="C18" s="32" t="s">
         <v>28</v>
@@ -2100,7 +2100,7 @@
       <c r="M18" s="11"/>
       <c r="N18" s="20"/>
     </row>
-    <row r="19" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="9"/>
       <c r="C19" s="22"/>
       <c r="D19" s="22"/>
@@ -2109,7 +2109,7 @@
       <c r="M19" s="11"/>
       <c r="N19" s="20"/>
     </row>
-    <row r="20" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="9"/>
       <c r="C20" s="28" t="s">
         <v>49</v>
@@ -2124,7 +2124,7 @@
       <c r="M20" s="11"/>
       <c r="N20" s="20"/>
     </row>
-    <row r="21" spans="2:14" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" ht="11.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="9"/>
       <c r="C21" s="29" t="s">
         <v>13</v>
@@ -2143,7 +2143,7 @@
       <c r="M21" s="11"/>
       <c r="N21" s="20"/>
     </row>
-    <row r="22" spans="2:14" ht="11.1" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:14" ht="11.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B22" s="9"/>
       <c r="C22" s="9" t="s">
         <v>48</v>
@@ -2158,7 +2158,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="9"/>
       <c r="C23" s="31" t="s">
         <v>38</v>
@@ -2172,7 +2172,7 @@
       <c r="M23" s="11"/>
       <c r="N23" s="20"/>
     </row>
-    <row r="24" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="9"/>
       <c r="C24" s="31" t="s">
         <v>39</v>
@@ -2193,7 +2193,7 @@
       <c r="M24" s="11"/>
       <c r="N24" s="20"/>
     </row>
-    <row r="25" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="9"/>
       <c r="C25" s="31" t="s">
         <v>42</v>
@@ -2207,7 +2207,7 @@
       <c r="M25" s="11"/>
       <c r="N25" s="20"/>
     </row>
-    <row r="26" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="9"/>
       <c r="C26" s="9" t="s">
         <v>43</v>
@@ -2228,7 +2228,7 @@
       <c r="M26" s="11"/>
       <c r="N26" s="20"/>
     </row>
-    <row r="27" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="9"/>
       <c r="C27" s="9" t="s">
         <v>19</v>
@@ -2243,7 +2243,7 @@
       <c r="M27" s="11"/>
       <c r="N27" s="20"/>
     </row>
-    <row r="28" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="9"/>
       <c r="C28" s="9" t="s">
         <v>20</v>
@@ -2261,7 +2261,7 @@
       <c r="M28" s="11"/>
       <c r="N28" s="20"/>
     </row>
-    <row r="29" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="9"/>
       <c r="C29" s="9" t="s">
         <v>21</v>
@@ -2274,7 +2274,7 @@
       <c r="M29" s="11"/>
       <c r="N29" s="20"/>
     </row>
-    <row r="30" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="9"/>
       <c r="C30" s="32" t="s">
         <v>28</v>
@@ -2294,107 +2294,107 @@
       <c r="M30" s="11"/>
       <c r="N30" s="20"/>
     </row>
-    <row r="31" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="9"/>
       <c r="L31" s="22"/>
       <c r="M31" s="11"/>
       <c r="N31" s="20"/>
     </row>
-    <row r="32" spans="2:14" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:14" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="9"/>
       <c r="L32" s="22"/>
       <c r="M32" s="11"/>
     </row>
-    <row r="33" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="9"/>
       <c r="L33" s="22"/>
       <c r="M33" s="11"/>
     </row>
-    <row r="34" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="9"/>
       <c r="L34" s="22"/>
       <c r="M34" s="11"/>
     </row>
-    <row r="35" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="9"/>
       <c r="L35" s="22"/>
       <c r="M35" s="11"/>
     </row>
-    <row r="36" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="9"/>
       <c r="L36" s="22"/>
       <c r="M36" s="11"/>
     </row>
-    <row r="37" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="9"/>
       <c r="L37" s="22"/>
       <c r="M37" s="11"/>
     </row>
-    <row r="38" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="9"/>
       <c r="L38" s="22"/>
       <c r="M38" s="11"/>
     </row>
-    <row r="39" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="9"/>
       <c r="L39" s="22"/>
       <c r="M39" s="11"/>
     </row>
-    <row r="40" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="9"/>
       <c r="L40" s="22"/>
       <c r="M40" s="11"/>
     </row>
-    <row r="41" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="9"/>
       <c r="L41" s="22"/>
       <c r="M41" s="11"/>
     </row>
-    <row r="42" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="9"/>
       <c r="M42" s="11"/>
     </row>
-    <row r="43" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="9"/>
       <c r="M43" s="11"/>
     </row>
-    <row r="44" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="9"/>
       <c r="M44" s="11"/>
     </row>
-    <row r="45" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="9"/>
       <c r="M45" s="11"/>
     </row>
-    <row r="46" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="9"/>
       <c r="M46" s="11"/>
     </row>
-    <row r="47" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="9"/>
       <c r="M47" s="11"/>
     </row>
-    <row r="48" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="9"/>
       <c r="M48" s="11"/>
     </row>
-    <row r="49" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="9"/>
       <c r="M49" s="11"/>
     </row>
-    <row r="50" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="9"/>
       <c r="M50" s="11"/>
     </row>
-    <row r="51" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="9"/>
       <c r="M51" s="11"/>
     </row>
-    <row r="52" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B52" s="9"/>
       <c r="M52" s="11"/>
     </row>
-    <row r="53" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
       <c r="D53" s="15"/>
@@ -2408,62 +2408,62 @@
       <c r="L53" s="15"/>
       <c r="M53" s="17"/>
     </row>
-    <row r="54" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="55" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="61" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="62" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="63" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="64" spans="2:13" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="65" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="67" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="68" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="69" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="70" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="73" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="74" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="76" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="77" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="78" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="80" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="81" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="82" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="83" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="85" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="87" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="89" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="90" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="91" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="92" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="94" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="103" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="104" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="105" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="106" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="107" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="108" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="109" ht="11.1" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="54" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="2:13" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="81" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="83" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="84" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" ht="11.15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection formatCells="0" insertHyperlinks="0" sort="0" autoFilter="0" pivotTables="0"/>
   <conditionalFormatting sqref="L1">

</xml_diff>